<commit_message>
Update migration artifacts for adventures pages
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adventures-listing.report.xlsx
+++ b/tools/importer/reports/import-adventures-listing.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
   <si>
     <t>_reportFile</t>
   </si>
@@ -73,13 +73,64 @@
     <t>adventures-listing</t>
   </si>
   <si>
-    <t>2026-07-23T10:43:12.588Z</t>
+    <t>2026-07-23T10:48:53.507Z</t>
   </si>
   <si>
     <t>Adventures</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp.report.json</t>
+  </si>
+  <si>
+    <t>["breadcrumb","hero","info-panel","tabs"]</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp</t>
+  </si>
+  <si>
+    <t>adventure-detail</t>
+  </si>
+  <si>
+    <t>2026-07-23T10:43:16.349Z</t>
+  </si>
+  <si>
+    <t>Bali Surf Camp</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/bali-surf-camp.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/tahoe-skiing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/tahoe-skiing</t>
+  </si>
+  <si>
+    <t>2026-07-23T10:43:26.047Z</t>
+  </si>
+  <si>
+    <t>Tahoe Skiing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/tahoe-skiing.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/yosemite-backpacking.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/yosemite-backpacking</t>
+  </si>
+  <si>
+    <t>2026-07-23T10:43:20.906Z</t>
+  </si>
+  <si>
+    <t>Yosemite Backpacking</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/yosemite-backpacking.html</t>
   </si>
 </sst>
 </file>
@@ -468,16 +519,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="1" max="2" width="50" customWidth="1"/>
+    <col min="3" max="3" width="39" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="28" customWidth="1"/>
-    <col min="8" max="8" width="41" customWidth="1"/>
+    <col min="8" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -556,6 +606,84 @@
       </c>
       <c r="H3" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>